<commit_message>
Resultats RAGAS finaux — GPT-4o sur CTI-ATTACK (229 requetes)
context_recall=0.4192, context_precision=0.2416
answer_relevancy=0.2455, noise_sensitivity=0.0126

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/RAG-evaluation-results-final.xlsx
+++ b/RAG-evaluation-results-final.xlsx
@@ -459,7 +459,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>noise_sensitivity</t>
+          <t>noise_sensitivity(mode=relevant)</t>
         </is>
       </c>
     </row>
@@ -495,8 +495,12 @@
       <c r="G2" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
+      <c r="H2" t="n">
+        <v>0.3959231804815469</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -530,8 +534,12 @@
       <c r="G3" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
+      <c r="H3" t="n">
+        <v>0.3983712735234055</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -565,8 +573,12 @@
       <c r="G4" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
+      <c r="H4" t="n">
+        <v>0.3346747525098469</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -600,8 +612,12 @@
       <c r="G5" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -635,8 +651,12 @@
       <c r="G6" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
+      <c r="H6" t="n">
+        <v>0.3573957462489742</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -670,8 +690,12 @@
       <c r="G7" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
+      <c r="H7" t="n">
+        <v>0.3384626042592127</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -705,8 +729,12 @@
       <c r="G8" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
+      <c r="H8" t="n">
+        <v>0.3233876420006027</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -740,8 +768,12 @@
       <c r="G9" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
+      <c r="H9" t="n">
+        <v>0.3729415638982641</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -775,8 +807,12 @@
       <c r="G10" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
+      <c r="H10" t="n">
+        <v>0.3490925044452693</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -810,8 +846,12 @@
       <c r="G11" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -845,8 +885,12 @@
       <c r="G12" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
+      <c r="H12" t="n">
+        <v>0.337214975235425</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -880,8 +924,12 @@
       <c r="G13" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
+      <c r="H13" t="n">
+        <v>0.2904087153482441</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -915,8 +963,12 @@
       <c r="G14" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
+      <c r="H14" t="n">
+        <v>0.3919879841554654</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -950,8 +1002,12 @@
       <c r="G15" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
+      <c r="H15" t="n">
+        <v>0.3230449312129807</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -985,8 +1041,12 @@
       <c r="G16" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
+      <c r="H16" t="n">
+        <v>0.3271162665110795</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1020,8 +1080,12 @@
       <c r="G17" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
+      <c r="H17" t="n">
+        <v>0.33445366085103</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1055,8 +1119,12 @@
       <c r="G18" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
+      <c r="H18" t="n">
+        <v>0.3194615699209492</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1090,8 +1158,12 @@
       <c r="G19" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
+      <c r="H19" t="n">
+        <v>0.2526470374911879</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1125,8 +1197,12 @@
       <c r="G20" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1160,8 +1236,12 @@
       <c r="G21" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
+      <c r="H21" t="n">
+        <v>0.4494440395910261</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1195,8 +1275,12 @@
       <c r="G22" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
+      <c r="H22" t="n">
+        <v>0.4712192788822681</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1230,8 +1314,12 @@
       <c r="G23" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1265,8 +1353,12 @@
       <c r="G24" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
+      <c r="H24" t="n">
+        <v>0.4101083094645099</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1300,8 +1392,12 @@
       <c r="G25" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
+      <c r="H25" t="n">
+        <v>0.2600556483994439</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1335,8 +1431,12 @@
       <c r="G26" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
+      <c r="H26" t="n">
+        <v>0.361573055052403</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1370,8 +1470,12 @@
       <c r="G27" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1405,8 +1509,12 @@
       <c r="G28" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1440,8 +1548,12 @@
       <c r="G29" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
+      <c r="H29" t="n">
+        <v>0.3355557607072217</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1475,8 +1587,12 @@
       <c r="G30" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1510,8 +1626,12 @@
       <c r="G31" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
+      <c r="H31" t="n">
+        <v>0.3844098816736704</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1545,8 +1665,12 @@
       <c r="G32" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
+      <c r="H32" t="n">
+        <v>0.3726316338106974</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1580,8 +1704,12 @@
       <c r="G33" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
+      <c r="H33" t="n">
+        <v>0.3309029518389979</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1615,8 +1743,12 @@
       <c r="G34" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
+      <c r="H34" t="n">
+        <v>0.3266867774749271</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1650,8 +1782,12 @@
       <c r="G35" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
+      <c r="H35" t="n">
+        <v>0.2746496369293423</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1685,8 +1821,12 @@
       <c r="G36" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
+      <c r="H36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1720,8 +1860,12 @@
       <c r="G37" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
+      <c r="H37" t="n">
+        <v>0.3304861194159487</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1755,8 +1899,12 @@
       <c r="G38" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
+      <c r="H38" t="n">
+        <v>0.3416669286694845</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1790,8 +1938,12 @@
       <c r="G39" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
+      <c r="H39" t="n">
+        <v>0.3334130117371659</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1825,8 +1977,12 @@
       <c r="G40" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
+      <c r="H40" t="n">
+        <v>0.3574025833914107</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1860,8 +2016,12 @@
       <c r="G41" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
+      <c r="H41" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1891,7 +2051,9 @@
       <c r="G42" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H42" t="inlineStr"/>
+      <c r="H42" t="n">
+        <v>0</v>
+      </c>
       <c r="I42" t="inlineStr"/>
     </row>
     <row r="43">
@@ -1922,7 +2084,9 @@
       <c r="G43" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H43" t="inlineStr"/>
+      <c r="H43" t="n">
+        <v>0</v>
+      </c>
       <c r="I43" t="inlineStr"/>
     </row>
     <row r="44">
@@ -1957,8 +2121,12 @@
       <c r="G44" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
+      <c r="H44" t="n">
+        <v>0.3465014290631855</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1992,8 +2160,12 @@
       <c r="G45" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
+      <c r="H45" t="n">
+        <v>0.4378884914273083</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2027,8 +2199,12 @@
       <c r="G46" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
+      <c r="H46" t="n">
+        <v>0.2969308488586125</v>
+      </c>
+      <c r="I46" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2062,8 +2238,12 @@
       <c r="G47" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
+      <c r="H47" t="n">
+        <v>0.2404359460370922</v>
+      </c>
+      <c r="I47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2097,8 +2277,12 @@
       <c r="G48" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
+      <c r="H48" t="n">
+        <v>0.3398954342960795</v>
+      </c>
+      <c r="I48" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2132,8 +2316,12 @@
       <c r="G49" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
+      <c r="H49" t="n">
+        <v>0.3280497228023961</v>
+      </c>
+      <c r="I49" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2167,8 +2355,12 @@
       <c r="G50" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr"/>
+      <c r="H50" t="n">
+        <v>0.3469066840509311</v>
+      </c>
+      <c r="I50" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2202,8 +2394,12 @@
       <c r="G51" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
+      <c r="H51" t="n">
+        <v>0.4270362866950459</v>
+      </c>
+      <c r="I51" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2237,8 +2433,12 @@
       <c r="G52" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr"/>
+      <c r="H52" t="n">
+        <v>0.3338846198426777</v>
+      </c>
+      <c r="I52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2272,8 +2472,12 @@
       <c r="G53" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
+      <c r="H53" t="n">
+        <v>0.334799812950488</v>
+      </c>
+      <c r="I53" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2307,8 +2511,12 @@
       <c r="G54" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
+      <c r="H54" t="n">
+        <v>0.2645429437347809</v>
+      </c>
+      <c r="I54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2342,8 +2550,12 @@
       <c r="G55" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
+      <c r="H55" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2377,8 +2589,12 @@
       <c r="G56" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
+      <c r="H56" t="n">
+        <v>0.2634213060518316</v>
+      </c>
+      <c r="I56" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2412,8 +2628,12 @@
       <c r="G57" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
+      <c r="H57" t="n">
+        <v>0.3666826104365673</v>
+      </c>
+      <c r="I57" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2447,8 +2667,12 @@
       <c r="G58" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr"/>
+      <c r="H58" t="n">
+        <v>0</v>
+      </c>
+      <c r="I58" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2482,8 +2706,12 @@
       <c r="G59" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
+      <c r="H59" t="n">
+        <v>0.354557835495258</v>
+      </c>
+      <c r="I59" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2517,8 +2745,12 @@
       <c r="G60" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
+      <c r="H60" t="n">
+        <v>0.3398630230648827</v>
+      </c>
+      <c r="I60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2552,8 +2784,12 @@
       <c r="G61" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
+      <c r="H61" t="n">
+        <v>0.3400302096659954</v>
+      </c>
+      <c r="I61" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2587,8 +2823,12 @@
       <c r="G62" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
+      <c r="H62" t="n">
+        <v>0</v>
+      </c>
+      <c r="I62" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2622,8 +2862,12 @@
       <c r="G63" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
+      <c r="H63" t="n">
+        <v>0</v>
+      </c>
+      <c r="I63" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2657,8 +2901,12 @@
       <c r="G64" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H64" t="inlineStr"/>
-      <c r="I64" t="inlineStr"/>
+      <c r="H64" t="n">
+        <v>0.3227949018366925</v>
+      </c>
+      <c r="I64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2692,8 +2940,12 @@
       <c r="G65" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr"/>
+      <c r="H65" t="n">
+        <v>0.3662328426208824</v>
+      </c>
+      <c r="I65" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2727,8 +2979,12 @@
       <c r="G66" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr"/>
+      <c r="H66" t="n">
+        <v>0</v>
+      </c>
+      <c r="I66" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2762,8 +3018,12 @@
       <c r="G67" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H67" t="inlineStr"/>
-      <c r="I67" t="inlineStr"/>
+      <c r="H67" t="n">
+        <v>0.3129327701255819</v>
+      </c>
+      <c r="I67" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2797,8 +3057,12 @@
       <c r="G68" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H68" t="inlineStr"/>
-      <c r="I68" t="inlineStr"/>
+      <c r="H68" t="n">
+        <v>0</v>
+      </c>
+      <c r="I68" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2832,8 +3096,12 @@
       <c r="G69" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H69" t="inlineStr"/>
-      <c r="I69" t="inlineStr"/>
+      <c r="H69" t="n">
+        <v>0.2804175124639266</v>
+      </c>
+      <c r="I69" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2867,8 +3135,12 @@
       <c r="G70" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H70" t="inlineStr"/>
-      <c r="I70" t="inlineStr"/>
+      <c r="H70" t="n">
+        <v>0.264411389817085</v>
+      </c>
+      <c r="I70" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2902,8 +3174,12 @@
       <c r="G71" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H71" t="inlineStr"/>
-      <c r="I71" t="inlineStr"/>
+      <c r="H71" t="n">
+        <v>0.3380460794138952</v>
+      </c>
+      <c r="I71" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2937,8 +3213,12 @@
       <c r="G72" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H72" t="inlineStr"/>
-      <c r="I72" t="inlineStr"/>
+      <c r="H72" t="n">
+        <v>0.3263852928505339</v>
+      </c>
+      <c r="I72" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2972,8 +3252,12 @@
       <c r="G73" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H73" t="inlineStr"/>
-      <c r="I73" t="inlineStr"/>
+      <c r="H73" t="n">
+        <v>0</v>
+      </c>
+      <c r="I73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3007,8 +3291,12 @@
       <c r="G74" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H74" t="inlineStr"/>
-      <c r="I74" t="inlineStr"/>
+      <c r="H74" t="n">
+        <v>0</v>
+      </c>
+      <c r="I74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3042,8 +3330,12 @@
       <c r="G75" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H75" t="inlineStr"/>
-      <c r="I75" t="inlineStr"/>
+      <c r="H75" t="n">
+        <v>0.3956603588168276</v>
+      </c>
+      <c r="I75" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3077,8 +3369,12 @@
       <c r="G76" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H76" t="inlineStr"/>
-      <c r="I76" t="inlineStr"/>
+      <c r="H76" t="n">
+        <v>0.3683431941687839</v>
+      </c>
+      <c r="I76" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3112,8 +3408,12 @@
       <c r="G77" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H77" t="inlineStr"/>
-      <c r="I77" t="inlineStr"/>
+      <c r="H77" t="n">
+        <v>0.3858377330069981</v>
+      </c>
+      <c r="I77" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3147,8 +3447,12 @@
       <c r="G78" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H78" t="inlineStr"/>
-      <c r="I78" t="inlineStr"/>
+      <c r="H78" t="n">
+        <v>0.3602503366424042</v>
+      </c>
+      <c r="I78" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3182,8 +3486,12 @@
       <c r="G79" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H79" t="inlineStr"/>
-      <c r="I79" t="inlineStr"/>
+      <c r="H79" t="n">
+        <v>0.3645864394214559</v>
+      </c>
+      <c r="I79" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3217,8 +3525,12 @@
       <c r="G80" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H80" t="inlineStr"/>
-      <c r="I80" t="inlineStr"/>
+      <c r="H80" t="n">
+        <v>0</v>
+      </c>
+      <c r="I80" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -3252,8 +3564,12 @@
       <c r="G81" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H81" t="inlineStr"/>
-      <c r="I81" t="inlineStr"/>
+      <c r="H81" t="n">
+        <v>0.3378391811400992</v>
+      </c>
+      <c r="I81" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -3287,8 +3603,12 @@
       <c r="G82" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H82" t="inlineStr"/>
-      <c r="I82" t="inlineStr"/>
+      <c r="H82" t="n">
+        <v>0.3491521695370525</v>
+      </c>
+      <c r="I82" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -3322,8 +3642,12 @@
       <c r="G83" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H83" t="inlineStr"/>
-      <c r="I83" t="inlineStr"/>
+      <c r="H83" t="n">
+        <v>0.388175631991857</v>
+      </c>
+      <c r="I83" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3357,8 +3681,12 @@
       <c r="G84" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H84" t="inlineStr"/>
-      <c r="I84" t="inlineStr"/>
+      <c r="H84" t="n">
+        <v>0</v>
+      </c>
+      <c r="I84" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -3392,8 +3720,12 @@
       <c r="G85" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H85" t="inlineStr"/>
-      <c r="I85" t="inlineStr"/>
+      <c r="H85" t="n">
+        <v>0.2643552927793187</v>
+      </c>
+      <c r="I85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -3427,8 +3759,12 @@
       <c r="G86" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H86" t="inlineStr"/>
-      <c r="I86" t="inlineStr"/>
+      <c r="H86" t="n">
+        <v>0</v>
+      </c>
+      <c r="I86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3462,8 +3798,12 @@
       <c r="G87" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H87" t="inlineStr"/>
-      <c r="I87" t="inlineStr"/>
+      <c r="H87" t="n">
+        <v>0</v>
+      </c>
+      <c r="I87" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3497,8 +3837,12 @@
       <c r="G88" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H88" t="inlineStr"/>
-      <c r="I88" t="inlineStr"/>
+      <c r="H88" t="n">
+        <v>0.2842707048389556</v>
+      </c>
+      <c r="I88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3532,8 +3876,12 @@
       <c r="G89" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H89" t="inlineStr"/>
-      <c r="I89" t="inlineStr"/>
+      <c r="H89" t="n">
+        <v>0.4349872822833479</v>
+      </c>
+      <c r="I89" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -3567,8 +3915,12 @@
       <c r="G90" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H90" t="inlineStr"/>
-      <c r="I90" t="inlineStr"/>
+      <c r="H90" t="n">
+        <v>0.3510059458957699</v>
+      </c>
+      <c r="I90" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -3602,8 +3954,12 @@
       <c r="G91" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H91" t="inlineStr"/>
-      <c r="I91" t="inlineStr"/>
+      <c r="H91" t="n">
+        <v>0.3235713768540716</v>
+      </c>
+      <c r="I91" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3637,8 +3993,12 @@
       <c r="G92" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H92" t="inlineStr"/>
-      <c r="I92" t="inlineStr"/>
+      <c r="H92" t="n">
+        <v>0.4067830631576485</v>
+      </c>
+      <c r="I92" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3672,8 +4032,12 @@
       <c r="G93" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H93" t="inlineStr"/>
-      <c r="I93" t="inlineStr"/>
+      <c r="H93" t="n">
+        <v>0.3452930361635712</v>
+      </c>
+      <c r="I93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -3707,8 +4071,12 @@
       <c r="G94" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H94" t="inlineStr"/>
-      <c r="I94" t="inlineStr"/>
+      <c r="H94" t="n">
+        <v>0.370667359125326</v>
+      </c>
+      <c r="I94" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -3742,8 +4110,12 @@
       <c r="G95" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H95" t="inlineStr"/>
-      <c r="I95" t="inlineStr"/>
+      <c r="H95" t="n">
+        <v>0.3338181482796754</v>
+      </c>
+      <c r="I95" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -3777,8 +4149,12 @@
       <c r="G96" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H96" t="inlineStr"/>
-      <c r="I96" t="inlineStr"/>
+      <c r="H96" t="n">
+        <v>0</v>
+      </c>
+      <c r="I96" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -3812,8 +4188,12 @@
       <c r="G97" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H97" t="inlineStr"/>
-      <c r="I97" t="inlineStr"/>
+      <c r="H97" t="n">
+        <v>0.2814412638081423</v>
+      </c>
+      <c r="I97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3847,8 +4227,12 @@
       <c r="G98" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H98" t="inlineStr"/>
-      <c r="I98" t="inlineStr"/>
+      <c r="H98" t="n">
+        <v>0.3160711846218169</v>
+      </c>
+      <c r="I98" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3882,8 +4266,12 @@
       <c r="G99" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H99" t="inlineStr"/>
-      <c r="I99" t="inlineStr"/>
+      <c r="H99" t="n">
+        <v>0.20474573470237</v>
+      </c>
+      <c r="I99" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -3917,8 +4305,12 @@
       <c r="G100" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H100" t="inlineStr"/>
-      <c r="I100" t="inlineStr"/>
+      <c r="H100" t="n">
+        <v>0.2550928094696763</v>
+      </c>
+      <c r="I100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -3952,8 +4344,12 @@
       <c r="G101" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H101" t="inlineStr"/>
-      <c r="I101" t="inlineStr"/>
+      <c r="H101" t="n">
+        <v>0.3704346554103848</v>
+      </c>
+      <c r="I101" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -3987,8 +4383,12 @@
       <c r="G102" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H102" t="inlineStr"/>
-      <c r="I102" t="inlineStr"/>
+      <c r="H102" t="n">
+        <v>0.3408817777974017</v>
+      </c>
+      <c r="I102" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -4022,8 +4422,12 @@
       <c r="G103" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H103" t="inlineStr"/>
-      <c r="I103" t="inlineStr"/>
+      <c r="H103" t="n">
+        <v>0.2428822585379302</v>
+      </c>
+      <c r="I103" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -4057,8 +4461,12 @@
       <c r="G104" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H104" t="inlineStr"/>
-      <c r="I104" t="inlineStr"/>
+      <c r="H104" t="n">
+        <v>0</v>
+      </c>
+      <c r="I104" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -4092,8 +4500,12 @@
       <c r="G105" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H105" t="inlineStr"/>
-      <c r="I105" t="inlineStr"/>
+      <c r="H105" t="n">
+        <v>0.3593402362303157</v>
+      </c>
+      <c r="I105" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -4127,8 +4539,12 @@
       <c r="G106" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H106" t="inlineStr"/>
-      <c r="I106" t="inlineStr"/>
+      <c r="H106" t="n">
+        <v>0.3583222124034637</v>
+      </c>
+      <c r="I106" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -4162,8 +4578,12 @@
       <c r="G107" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H107" t="inlineStr"/>
-      <c r="I107" t="inlineStr"/>
+      <c r="H107" t="n">
+        <v>0</v>
+      </c>
+      <c r="I107" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -4197,8 +4617,12 @@
       <c r="G108" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H108" t="inlineStr"/>
-      <c r="I108" t="inlineStr"/>
+      <c r="H108" t="n">
+        <v>0.3390480050590213</v>
+      </c>
+      <c r="I108" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -4232,8 +4656,12 @@
       <c r="G109" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H109" t="inlineStr"/>
-      <c r="I109" t="inlineStr"/>
+      <c r="H109" t="n">
+        <v>0.4188152966293376</v>
+      </c>
+      <c r="I109" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -4267,8 +4695,12 @@
       <c r="G110" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H110" t="inlineStr"/>
-      <c r="I110" t="inlineStr"/>
+      <c r="H110" t="n">
+        <v>0.3316374782503308</v>
+      </c>
+      <c r="I110" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -4302,8 +4734,12 @@
       <c r="G111" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H111" t="inlineStr"/>
-      <c r="I111" t="inlineStr"/>
+      <c r="H111" t="n">
+        <v>0.3480280564411122</v>
+      </c>
+      <c r="I111" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -4337,8 +4773,12 @@
       <c r="G112" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H112" t="inlineStr"/>
-      <c r="I112" t="inlineStr"/>
+      <c r="H112" t="n">
+        <v>0.3894740049771969</v>
+      </c>
+      <c r="I112" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -4372,8 +4812,12 @@
       <c r="G113" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H113" t="inlineStr"/>
-      <c r="I113" t="inlineStr"/>
+      <c r="H113" t="n">
+        <v>0.4244909090874014</v>
+      </c>
+      <c r="I113" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -4407,8 +4851,12 @@
       <c r="G114" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H114" t="inlineStr"/>
-      <c r="I114" t="inlineStr"/>
+      <c r="H114" t="n">
+        <v>0.39737778707126</v>
+      </c>
+      <c r="I114" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -4442,8 +4890,12 @@
       <c r="G115" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H115" t="inlineStr"/>
-      <c r="I115" t="inlineStr"/>
+      <c r="H115" t="n">
+        <v>0</v>
+      </c>
+      <c r="I115" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -4477,8 +4929,12 @@
       <c r="G116" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H116" t="inlineStr"/>
-      <c r="I116" t="inlineStr"/>
+      <c r="H116" t="n">
+        <v>0.3238769621343572</v>
+      </c>
+      <c r="I116" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -4512,8 +4968,12 @@
       <c r="G117" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H117" t="inlineStr"/>
-      <c r="I117" t="inlineStr"/>
+      <c r="H117" t="n">
+        <v>0.3363716955003596</v>
+      </c>
+      <c r="I117" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -4547,8 +5007,12 @@
       <c r="G118" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H118" t="inlineStr"/>
-      <c r="I118" t="inlineStr"/>
+      <c r="H118" t="n">
+        <v>0.3806594751721678</v>
+      </c>
+      <c r="I118" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -4582,8 +5046,12 @@
       <c r="G119" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H119" t="inlineStr"/>
-      <c r="I119" t="inlineStr"/>
+      <c r="H119" t="n">
+        <v>0.3311630601235688</v>
+      </c>
+      <c r="I119" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -4617,8 +5085,12 @@
       <c r="G120" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H120" t="inlineStr"/>
-      <c r="I120" t="inlineStr"/>
+      <c r="H120" t="n">
+        <v>0</v>
+      </c>
+      <c r="I120" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -4652,8 +5124,12 @@
       <c r="G121" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H121" t="inlineStr"/>
-      <c r="I121" t="inlineStr"/>
+      <c r="H121" t="n">
+        <v>0.4164335389621195</v>
+      </c>
+      <c r="I121" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -4687,8 +5163,12 @@
       <c r="G122" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H122" t="inlineStr"/>
-      <c r="I122" t="inlineStr"/>
+      <c r="H122" t="n">
+        <v>0.3408577896721949</v>
+      </c>
+      <c r="I122" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -4722,8 +5202,12 @@
       <c r="G123" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H123" t="inlineStr"/>
-      <c r="I123" t="inlineStr"/>
+      <c r="H123" t="n">
+        <v>0.2917838972725384</v>
+      </c>
+      <c r="I123" t="n">
+        <v>0.3333333333333333</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -4757,8 +5241,12 @@
       <c r="G124" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H124" t="inlineStr"/>
-      <c r="I124" t="inlineStr"/>
+      <c r="H124" t="n">
+        <v>0.3737171112132614</v>
+      </c>
+      <c r="I124" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -4792,8 +5280,12 @@
       <c r="G125" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H125" t="inlineStr"/>
-      <c r="I125" t="inlineStr"/>
+      <c r="H125" t="n">
+        <v>0.341152492380347</v>
+      </c>
+      <c r="I125" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -4827,8 +5319,12 @@
       <c r="G126" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H126" t="inlineStr"/>
-      <c r="I126" t="inlineStr"/>
+      <c r="H126" t="n">
+        <v>0.3167462649623461</v>
+      </c>
+      <c r="I126" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -4862,8 +5358,12 @@
       <c r="G127" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H127" t="inlineStr"/>
-      <c r="I127" t="inlineStr"/>
+      <c r="H127" t="n">
+        <v>0.3753104794365369</v>
+      </c>
+      <c r="I127" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -4897,8 +5397,12 @@
       <c r="G128" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H128" t="inlineStr"/>
-      <c r="I128" t="inlineStr"/>
+      <c r="H128" t="n">
+        <v>0</v>
+      </c>
+      <c r="I128" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -4932,8 +5436,12 @@
       <c r="G129" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H129" t="inlineStr"/>
-      <c r="I129" t="inlineStr"/>
+      <c r="H129" t="n">
+        <v>0.3311062076986086</v>
+      </c>
+      <c r="I129" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -4967,8 +5475,12 @@
       <c r="G130" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H130" t="inlineStr"/>
-      <c r="I130" t="inlineStr"/>
+      <c r="H130" t="n">
+        <v>0.3520635984473916</v>
+      </c>
+      <c r="I130" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -5002,8 +5514,12 @@
       <c r="G131" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H131" t="inlineStr"/>
-      <c r="I131" t="inlineStr"/>
+      <c r="H131" t="n">
+        <v>0.185800742147395</v>
+      </c>
+      <c r="I131" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -5037,8 +5553,12 @@
       <c r="G132" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H132" t="inlineStr"/>
-      <c r="I132" t="inlineStr"/>
+      <c r="H132" t="n">
+        <v>0.3396766372787157</v>
+      </c>
+      <c r="I132" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -5072,8 +5592,12 @@
       <c r="G133" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H133" t="inlineStr"/>
-      <c r="I133" t="inlineStr"/>
+      <c r="H133" t="n">
+        <v>0.3778358123556588</v>
+      </c>
+      <c r="I133" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -5107,8 +5631,12 @@
       <c r="G134" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H134" t="inlineStr"/>
-      <c r="I134" t="inlineStr"/>
+      <c r="H134" t="n">
+        <v>0</v>
+      </c>
+      <c r="I134" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -5142,8 +5670,12 @@
       <c r="G135" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H135" t="inlineStr"/>
-      <c r="I135" t="inlineStr"/>
+      <c r="H135" t="n">
+        <v>0.3254713638849845</v>
+      </c>
+      <c r="I135" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -5177,8 +5709,12 @@
       <c r="G136" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H136" t="inlineStr"/>
-      <c r="I136" t="inlineStr"/>
+      <c r="H136" t="n">
+        <v>0</v>
+      </c>
+      <c r="I136" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -5212,8 +5748,12 @@
       <c r="G137" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H137" t="inlineStr"/>
-      <c r="I137" t="inlineStr"/>
+      <c r="H137" t="n">
+        <v>0.4238381322568959</v>
+      </c>
+      <c r="I137" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -5247,8 +5787,12 @@
       <c r="G138" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H138" t="inlineStr"/>
-      <c r="I138" t="inlineStr"/>
+      <c r="H138" t="n">
+        <v>0.4165724544343138</v>
+      </c>
+      <c r="I138" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -5282,8 +5826,12 @@
       <c r="G139" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H139" t="inlineStr"/>
-      <c r="I139" t="inlineStr"/>
+      <c r="H139" t="n">
+        <v>0</v>
+      </c>
+      <c r="I139" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -5317,8 +5865,12 @@
       <c r="G140" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H140" t="inlineStr"/>
-      <c r="I140" t="inlineStr"/>
+      <c r="H140" t="n">
+        <v>0.3205968771138361</v>
+      </c>
+      <c r="I140" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -5352,8 +5904,12 @@
       <c r="G141" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H141" t="inlineStr"/>
-      <c r="I141" t="inlineStr"/>
+      <c r="H141" t="n">
+        <v>0</v>
+      </c>
+      <c r="I141" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -5387,8 +5943,12 @@
       <c r="G142" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H142" t="inlineStr"/>
-      <c r="I142" t="inlineStr"/>
+      <c r="H142" t="n">
+        <v>0.3278974152609673</v>
+      </c>
+      <c r="I142" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -5422,8 +5982,12 @@
       <c r="G143" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H143" t="inlineStr"/>
-      <c r="I143" t="inlineStr"/>
+      <c r="H143" t="n">
+        <v>0</v>
+      </c>
+      <c r="I143" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -5457,8 +6021,12 @@
       <c r="G144" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H144" t="inlineStr"/>
-      <c r="I144" t="inlineStr"/>
+      <c r="H144" t="n">
+        <v>0</v>
+      </c>
+      <c r="I144" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -5492,8 +6060,12 @@
       <c r="G145" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H145" t="inlineStr"/>
-      <c r="I145" t="inlineStr"/>
+      <c r="H145" t="n">
+        <v>0.3447577654478497</v>
+      </c>
+      <c r="I145" t="n">
+        <v>0.25</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -5527,8 +6099,12 @@
       <c r="G146" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H146" t="inlineStr"/>
-      <c r="I146" t="inlineStr"/>
+      <c r="H146" t="n">
+        <v>0.4020332982747918</v>
+      </c>
+      <c r="I146" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -5562,8 +6138,12 @@
       <c r="G147" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H147" t="inlineStr"/>
-      <c r="I147" t="inlineStr"/>
+      <c r="H147" t="n">
+        <v>0.333367040819245</v>
+      </c>
+      <c r="I147" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -5597,8 +6177,12 @@
       <c r="G148" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H148" t="inlineStr"/>
-      <c r="I148" t="inlineStr"/>
+      <c r="H148" t="n">
+        <v>0.4259819397933462</v>
+      </c>
+      <c r="I148" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -5632,8 +6216,12 @@
       <c r="G149" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H149" t="inlineStr"/>
-      <c r="I149" t="inlineStr"/>
+      <c r="H149" t="n">
+        <v>0.3338197389751817</v>
+      </c>
+      <c r="I149" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -5667,8 +6255,12 @@
       <c r="G150" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H150" t="inlineStr"/>
-      <c r="I150" t="inlineStr"/>
+      <c r="H150" t="n">
+        <v>0.360140798190365</v>
+      </c>
+      <c r="I150" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -5702,8 +6294,12 @@
       <c r="G151" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H151" t="inlineStr"/>
-      <c r="I151" t="inlineStr"/>
+      <c r="H151" t="n">
+        <v>0.2405044917227062</v>
+      </c>
+      <c r="I151" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -5737,8 +6333,12 @@
       <c r="G152" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H152" t="inlineStr"/>
-      <c r="I152" t="inlineStr"/>
+      <c r="H152" t="n">
+        <v>0</v>
+      </c>
+      <c r="I152" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -5772,8 +6372,12 @@
       <c r="G153" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H153" t="inlineStr"/>
-      <c r="I153" t="inlineStr"/>
+      <c r="H153" t="n">
+        <v>0</v>
+      </c>
+      <c r="I153" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -5807,8 +6411,12 @@
       <c r="G154" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H154" t="inlineStr"/>
-      <c r="I154" t="inlineStr"/>
+      <c r="H154" t="n">
+        <v>0.21578066794825</v>
+      </c>
+      <c r="I154" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -5842,8 +6450,12 @@
       <c r="G155" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H155" t="inlineStr"/>
-      <c r="I155" t="inlineStr"/>
+      <c r="H155" t="n">
+        <v>0.3374624415738935</v>
+      </c>
+      <c r="I155" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -5877,8 +6489,12 @@
       <c r="G156" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H156" t="inlineStr"/>
-      <c r="I156" t="inlineStr"/>
+      <c r="H156" t="n">
+        <v>0</v>
+      </c>
+      <c r="I156" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -5912,8 +6528,12 @@
       <c r="G157" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H157" t="inlineStr"/>
-      <c r="I157" t="inlineStr"/>
+      <c r="H157" t="n">
+        <v>0.3371751765725229</v>
+      </c>
+      <c r="I157" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -5947,8 +6567,12 @@
       <c r="G158" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H158" t="inlineStr"/>
-      <c r="I158" t="inlineStr"/>
+      <c r="H158" t="n">
+        <v>0.2200599979117083</v>
+      </c>
+      <c r="I158" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -5982,8 +6606,12 @@
       <c r="G159" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H159" t="inlineStr"/>
-      <c r="I159" t="inlineStr"/>
+      <c r="H159" t="n">
+        <v>0.3820331967820332</v>
+      </c>
+      <c r="I159" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -6017,8 +6645,12 @@
       <c r="G160" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H160" t="inlineStr"/>
-      <c r="I160" t="inlineStr"/>
+      <c r="H160" t="n">
+        <v>0</v>
+      </c>
+      <c r="I160" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -6052,8 +6684,12 @@
       <c r="G161" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H161" t="inlineStr"/>
-      <c r="I161" t="inlineStr"/>
+      <c r="H161" t="n">
+        <v>0.428442216353832</v>
+      </c>
+      <c r="I161" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -6087,8 +6723,12 @@
       <c r="G162" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H162" t="inlineStr"/>
-      <c r="I162" t="inlineStr"/>
+      <c r="H162" t="n">
+        <v>0.2992110916121975</v>
+      </c>
+      <c r="I162" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -6122,8 +6762,12 @@
       <c r="G163" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H163" t="inlineStr"/>
-      <c r="I163" t="inlineStr"/>
+      <c r="H163" t="n">
+        <v>0</v>
+      </c>
+      <c r="I163" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -6157,8 +6801,12 @@
       <c r="G164" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H164" t="inlineStr"/>
-      <c r="I164" t="inlineStr"/>
+      <c r="H164" t="n">
+        <v>0.3280616135639453</v>
+      </c>
+      <c r="I164" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -6192,8 +6840,12 @@
       <c r="G165" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H165" t="inlineStr"/>
-      <c r="I165" t="inlineStr"/>
+      <c r="H165" t="n">
+        <v>0</v>
+      </c>
+      <c r="I165" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -6227,8 +6879,12 @@
       <c r="G166" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H166" t="inlineStr"/>
-      <c r="I166" t="inlineStr"/>
+      <c r="H166" t="n">
+        <v>0.4993650633417702</v>
+      </c>
+      <c r="I166" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -6262,8 +6918,12 @@
       <c r="G167" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H167" t="inlineStr"/>
-      <c r="I167" t="inlineStr"/>
+      <c r="H167" t="n">
+        <v>0</v>
+      </c>
+      <c r="I167" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -6297,8 +6957,12 @@
       <c r="G168" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H168" t="inlineStr"/>
-      <c r="I168" t="inlineStr"/>
+      <c r="H168" t="n">
+        <v>0.3753071154244798</v>
+      </c>
+      <c r="I168" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -6332,8 +6996,12 @@
       <c r="G169" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H169" t="inlineStr"/>
-      <c r="I169" t="inlineStr"/>
+      <c r="H169" t="n">
+        <v>0.2708280509904981</v>
+      </c>
+      <c r="I169" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -6367,8 +7035,12 @@
       <c r="G170" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H170" t="inlineStr"/>
-      <c r="I170" t="inlineStr"/>
+      <c r="H170" t="n">
+        <v>0</v>
+      </c>
+      <c r="I170" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -6402,8 +7074,12 @@
       <c r="G171" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H171" t="inlineStr"/>
-      <c r="I171" t="inlineStr"/>
+      <c r="H171" t="n">
+        <v>0.3658465134271952</v>
+      </c>
+      <c r="I171" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -6437,8 +7113,12 @@
       <c r="G172" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H172" t="inlineStr"/>
-      <c r="I172" t="inlineStr"/>
+      <c r="H172" t="n">
+        <v>0.2608843265702252</v>
+      </c>
+      <c r="I172" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -6472,8 +7152,12 @@
       <c r="G173" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H173" t="inlineStr"/>
-      <c r="I173" t="inlineStr"/>
+      <c r="H173" t="n">
+        <v>0.3964741779320002</v>
+      </c>
+      <c r="I173" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -6507,8 +7191,12 @@
       <c r="G174" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H174" t="inlineStr"/>
-      <c r="I174" t="inlineStr"/>
+      <c r="H174" t="n">
+        <v>0.3443693183738757</v>
+      </c>
+      <c r="I174" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -6542,8 +7230,12 @@
       <c r="G175" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H175" t="inlineStr"/>
-      <c r="I175" t="inlineStr"/>
+      <c r="H175" t="n">
+        <v>0.2737579041780179</v>
+      </c>
+      <c r="I175" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -6577,8 +7269,12 @@
       <c r="G176" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H176" t="inlineStr"/>
-      <c r="I176" t="inlineStr"/>
+      <c r="H176" t="n">
+        <v>0</v>
+      </c>
+      <c r="I176" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -6612,8 +7308,12 @@
       <c r="G177" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H177" t="inlineStr"/>
-      <c r="I177" t="inlineStr"/>
+      <c r="H177" t="n">
+        <v>0.3432347430472884</v>
+      </c>
+      <c r="I177" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -6647,8 +7347,12 @@
       <c r="G178" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H178" t="inlineStr"/>
-      <c r="I178" t="inlineStr"/>
+      <c r="H178" t="n">
+        <v>0.3975512025859732</v>
+      </c>
+      <c r="I178" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -6682,8 +7386,12 @@
       <c r="G179" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H179" t="inlineStr"/>
-      <c r="I179" t="inlineStr"/>
+      <c r="H179" t="n">
+        <v>0.2639845357016807</v>
+      </c>
+      <c r="I179" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -6717,8 +7425,12 @@
       <c r="G180" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H180" t="inlineStr"/>
-      <c r="I180" t="inlineStr"/>
+      <c r="H180" t="n">
+        <v>0.2801281865629768</v>
+      </c>
+      <c r="I180" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -6752,8 +7464,12 @@
       <c r="G181" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H181" t="inlineStr"/>
-      <c r="I181" t="inlineStr"/>
+      <c r="H181" t="n">
+        <v>0</v>
+      </c>
+      <c r="I181" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -6787,8 +7503,12 @@
       <c r="G182" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H182" t="inlineStr"/>
-      <c r="I182" t="inlineStr"/>
+      <c r="H182" t="n">
+        <v>0.3366106858994586</v>
+      </c>
+      <c r="I182" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -6822,8 +7542,12 @@
       <c r="G183" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H183" t="inlineStr"/>
-      <c r="I183" t="inlineStr"/>
+      <c r="H183" t="n">
+        <v>0</v>
+      </c>
+      <c r="I183" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -6857,8 +7581,12 @@
       <c r="G184" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H184" t="inlineStr"/>
-      <c r="I184" t="inlineStr"/>
+      <c r="H184" t="n">
+        <v>0</v>
+      </c>
+      <c r="I184" t="n">
+        <v>0.25</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -6892,8 +7620,12 @@
       <c r="G185" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H185" t="inlineStr"/>
-      <c r="I185" t="inlineStr"/>
+      <c r="H185" t="n">
+        <v>0</v>
+      </c>
+      <c r="I185" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -6927,8 +7659,12 @@
       <c r="G186" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H186" t="inlineStr"/>
-      <c r="I186" t="inlineStr"/>
+      <c r="H186" t="n">
+        <v>0.3230229236986693</v>
+      </c>
+      <c r="I186" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -6962,8 +7698,12 @@
       <c r="G187" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H187" t="inlineStr"/>
-      <c r="I187" t="inlineStr"/>
+      <c r="H187" t="n">
+        <v>0</v>
+      </c>
+      <c r="I187" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -6997,8 +7737,12 @@
       <c r="G188" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H188" t="inlineStr"/>
-      <c r="I188" t="inlineStr"/>
+      <c r="H188" t="n">
+        <v>0.2267837370059973</v>
+      </c>
+      <c r="I188" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -7032,8 +7776,12 @@
       <c r="G189" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H189" t="inlineStr"/>
-      <c r="I189" t="inlineStr"/>
+      <c r="H189" t="n">
+        <v>0.4070186008600092</v>
+      </c>
+      <c r="I189" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -7067,8 +7815,12 @@
       <c r="G190" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H190" t="inlineStr"/>
-      <c r="I190" t="inlineStr"/>
+      <c r="H190" t="n">
+        <v>0</v>
+      </c>
+      <c r="I190" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -7102,8 +7854,12 @@
       <c r="G191" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H191" t="inlineStr"/>
-      <c r="I191" t="inlineStr"/>
+      <c r="H191" t="n">
+        <v>0.4454792052173761</v>
+      </c>
+      <c r="I191" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -7137,8 +7893,12 @@
       <c r="G192" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H192" t="inlineStr"/>
-      <c r="I192" t="inlineStr"/>
+      <c r="H192" t="n">
+        <v>0</v>
+      </c>
+      <c r="I192" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -7172,8 +7932,12 @@
       <c r="G193" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H193" t="inlineStr"/>
-      <c r="I193" t="inlineStr"/>
+      <c r="H193" t="n">
+        <v>0.3365897990682189</v>
+      </c>
+      <c r="I193" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -7207,8 +7971,12 @@
       <c r="G194" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H194" t="inlineStr"/>
-      <c r="I194" t="inlineStr"/>
+      <c r="H194" t="n">
+        <v>0</v>
+      </c>
+      <c r="I194" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -7242,8 +8010,12 @@
       <c r="G195" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H195" t="inlineStr"/>
-      <c r="I195" t="inlineStr"/>
+      <c r="H195" t="n">
+        <v>0.3355688236658207</v>
+      </c>
+      <c r="I195" t="n">
+        <v>0.25</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -7277,8 +8049,12 @@
       <c r="G196" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H196" t="inlineStr"/>
-      <c r="I196" t="inlineStr"/>
+      <c r="H196" t="n">
+        <v>0.3956570642034127</v>
+      </c>
+      <c r="I196" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -7312,8 +8088,12 @@
       <c r="G197" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H197" t="inlineStr"/>
-      <c r="I197" t="inlineStr"/>
+      <c r="H197" t="n">
+        <v>0.4075326100721035</v>
+      </c>
+      <c r="I197" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -7347,8 +8127,12 @@
       <c r="G198" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H198" t="inlineStr"/>
-      <c r="I198" t="inlineStr"/>
+      <c r="H198" t="n">
+        <v>0.3326972408957315</v>
+      </c>
+      <c r="I198" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -7378,7 +8162,9 @@
       <c r="G199" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H199" t="inlineStr"/>
+      <c r="H199" t="n">
+        <v>0</v>
+      </c>
       <c r="I199" t="inlineStr"/>
     </row>
     <row r="200">
@@ -7413,8 +8199,12 @@
       <c r="G200" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H200" t="inlineStr"/>
-      <c r="I200" t="inlineStr"/>
+      <c r="H200" t="n">
+        <v>0</v>
+      </c>
+      <c r="I200" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -7448,8 +8238,12 @@
       <c r="G201" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H201" t="inlineStr"/>
-      <c r="I201" t="inlineStr"/>
+      <c r="H201" t="n">
+        <v>0.3365897990682189</v>
+      </c>
+      <c r="I201" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -7483,8 +8277,12 @@
       <c r="G202" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H202" t="inlineStr"/>
-      <c r="I202" t="inlineStr"/>
+      <c r="H202" t="n">
+        <v>0</v>
+      </c>
+      <c r="I202" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -7518,8 +8316,12 @@
       <c r="G203" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H203" t="inlineStr"/>
-      <c r="I203" t="inlineStr"/>
+      <c r="H203" t="n">
+        <v>0</v>
+      </c>
+      <c r="I203" t="n">
+        <v>0.25</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -7553,8 +8355,12 @@
       <c r="G204" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H204" t="inlineStr"/>
-      <c r="I204" t="inlineStr"/>
+      <c r="H204" t="n">
+        <v>0.3291153802500701</v>
+      </c>
+      <c r="I204" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -7588,8 +8394,12 @@
       <c r="G205" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H205" t="inlineStr"/>
-      <c r="I205" t="inlineStr"/>
+      <c r="H205" t="n">
+        <v>0.4725444364995491</v>
+      </c>
+      <c r="I205" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -7623,8 +8433,12 @@
       <c r="G206" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H206" t="inlineStr"/>
-      <c r="I206" t="inlineStr"/>
+      <c r="H206" t="n">
+        <v>0.2483791660543884</v>
+      </c>
+      <c r="I206" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -7658,8 +8472,12 @@
       <c r="G207" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H207" t="inlineStr"/>
-      <c r="I207" t="inlineStr"/>
+      <c r="H207" t="n">
+        <v>0.3741827887951039</v>
+      </c>
+      <c r="I207" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -7693,8 +8511,12 @@
       <c r="G208" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H208" t="inlineStr"/>
-      <c r="I208" t="inlineStr"/>
+      <c r="H208" t="n">
+        <v>0.2624445527785361</v>
+      </c>
+      <c r="I208" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -7728,8 +8550,12 @@
       <c r="G209" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H209" t="inlineStr"/>
-      <c r="I209" t="inlineStr"/>
+      <c r="H209" t="n">
+        <v>0.3776370915845159</v>
+      </c>
+      <c r="I209" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -7763,8 +8589,12 @@
       <c r="G210" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H210" t="inlineStr"/>
-      <c r="I210" t="inlineStr"/>
+      <c r="H210" t="n">
+        <v>0</v>
+      </c>
+      <c r="I210" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -7798,8 +8628,12 @@
       <c r="G211" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H211" t="inlineStr"/>
-      <c r="I211" t="inlineStr"/>
+      <c r="H211" t="n">
+        <v>0</v>
+      </c>
+      <c r="I211" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -7833,8 +8667,12 @@
       <c r="G212" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H212" t="inlineStr"/>
-      <c r="I212" t="inlineStr"/>
+      <c r="H212" t="n">
+        <v>0.3436662014815008</v>
+      </c>
+      <c r="I212" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -7868,8 +8706,12 @@
       <c r="G213" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H213" t="inlineStr"/>
-      <c r="I213" t="inlineStr"/>
+      <c r="H213" t="n">
+        <v>0</v>
+      </c>
+      <c r="I213" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -7903,8 +8745,12 @@
       <c r="G214" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H214" t="inlineStr"/>
-      <c r="I214" t="inlineStr"/>
+      <c r="H214" t="n">
+        <v>0.4115095012629742</v>
+      </c>
+      <c r="I214" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -7934,7 +8780,9 @@
       <c r="G215" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H215" t="inlineStr"/>
+      <c r="H215" t="n">
+        <v>0</v>
+      </c>
       <c r="I215" t="inlineStr"/>
     </row>
     <row r="216">
@@ -7969,8 +8817,12 @@
       <c r="G216" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H216" t="inlineStr"/>
-      <c r="I216" t="inlineStr"/>
+      <c r="H216" t="n">
+        <v>0.3885963182077558</v>
+      </c>
+      <c r="I216" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -8004,8 +8856,12 @@
       <c r="G217" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H217" t="inlineStr"/>
-      <c r="I217" t="inlineStr"/>
+      <c r="H217" t="n">
+        <v>0.306674856594968</v>
+      </c>
+      <c r="I217" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -8039,8 +8895,12 @@
       <c r="G218" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H218" t="inlineStr"/>
-      <c r="I218" t="inlineStr"/>
+      <c r="H218" t="n">
+        <v>0.416967379625422</v>
+      </c>
+      <c r="I218" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -8070,7 +8930,9 @@
       <c r="G219" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H219" t="inlineStr"/>
+      <c r="H219" t="n">
+        <v>0</v>
+      </c>
       <c r="I219" t="inlineStr"/>
     </row>
     <row r="220">
@@ -8105,8 +8967,12 @@
       <c r="G220" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H220" t="inlineStr"/>
-      <c r="I220" t="inlineStr"/>
+      <c r="H220" t="n">
+        <v>0.3980351778479036</v>
+      </c>
+      <c r="I220" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -8140,8 +9006,12 @@
       <c r="G221" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H221" t="inlineStr"/>
-      <c r="I221" t="inlineStr"/>
+      <c r="H221" t="n">
+        <v>0.318229061294664</v>
+      </c>
+      <c r="I221" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -8175,8 +9045,12 @@
       <c r="G222" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H222" t="inlineStr"/>
-      <c r="I222" t="inlineStr"/>
+      <c r="H222" t="n">
+        <v>0.4229546407543196</v>
+      </c>
+      <c r="I222" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -8210,8 +9084,12 @@
       <c r="G223" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H223" t="inlineStr"/>
-      <c r="I223" t="inlineStr"/>
+      <c r="H223" t="n">
+        <v>0</v>
+      </c>
+      <c r="I223" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -8245,8 +9123,12 @@
       <c r="G224" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H224" t="inlineStr"/>
-      <c r="I224" t="inlineStr"/>
+      <c r="H224" t="n">
+        <v>0</v>
+      </c>
+      <c r="I224" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -8280,8 +9162,12 @@
       <c r="G225" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H225" t="inlineStr"/>
-      <c r="I225" t="inlineStr"/>
+      <c r="H225" t="n">
+        <v>0.4674683117646577</v>
+      </c>
+      <c r="I225" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -8315,8 +9201,12 @@
       <c r="G226" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H226" t="inlineStr"/>
-      <c r="I226" t="inlineStr"/>
+      <c r="H226" t="n">
+        <v>0.3386014966736512</v>
+      </c>
+      <c r="I226" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -8350,8 +9240,12 @@
       <c r="G227" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H227" t="inlineStr"/>
-      <c r="I227" t="inlineStr"/>
+      <c r="H227" t="n">
+        <v>0</v>
+      </c>
+      <c r="I227" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -8385,8 +9279,12 @@
       <c r="G228" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H228" t="inlineStr"/>
-      <c r="I228" t="inlineStr"/>
+      <c r="H228" t="n">
+        <v>0</v>
+      </c>
+      <c r="I228" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -8420,8 +9318,12 @@
       <c r="G229" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H229" t="inlineStr"/>
-      <c r="I229" t="inlineStr"/>
+      <c r="H229" t="n">
+        <v>0</v>
+      </c>
+      <c r="I229" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -8455,8 +9357,12 @@
       <c r="G230" t="n">
         <v>0.2416302765443231</v>
       </c>
-      <c r="H230" t="inlineStr"/>
-      <c r="I230" t="inlineStr"/>
+      <c r="H230" t="n">
+        <v>0.3675806981699321</v>
+      </c>
+      <c r="I230" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>